<commit_message>
Add columns-service, promo-card blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (14):
- blocks/columns-service/columns-service.css
- blocks/columns-service/_columns-service.json -> blocks/promo-card/_promo-card.json
- blocks/columns-service/metadata.json -> blocks/promo-card/metadata.json
- blocks/promo-card/promo-card.css
- blocks/columns-service/columns-service.js -> blocks/promo-card/promo-card.js
- component-definition.json
- component-filters.json
- component-models.json
- tools/importer/import-hey-conad.bundle.js
- tools/importer/import-hey-conad.js
- tools/importer/page-templates.json
- tools/importer/parsers/columns-service.js -> tools/importer/parsers/promo-card.js
- tools/importer/reports/hey-conad.report.json
- tools/importer/reports/import-hey-conad.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-hey-conad.report.xlsx
+++ b/tools/importer/reports/import-hey-conad.report.xlsx
@@ -40,7 +40,7 @@
     <t>hey-conad.report.json</t>
   </si>
   <si>
-    <t>["hero-landing","columns-banner","columns-service","columns-service","columns-service","columns-service"]</t>
+    <t>["hero-landing","columns-banner","promo-card","promo-card","promo-card","promo-card"]</t>
   </si>
   <si>
     <t>hey-conad</t>
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-05-26T16:32:37.397Z</t>
+    <t>2026-05-26T16:43:04.041Z</t>
   </si>
   <si>
     <t>Hey Conad | Scarica l’App | Acquista Online i nostri Servizi Digitali | Conad</t>

</xml_diff>

<commit_message>
Add columns-banner, cta-banner blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (17):
- blocks/columns-banner/_columns-banner.json
- blocks/columns-banner/columns-banner.js
- blocks/cta-banner/_cta-banner.json
- blocks/columns-banner/columns-banner.css -> blocks/cta-banner/cta-banner.css
- blocks/cta-banner/cta-banner.js
- blocks/columns-banner/metadata.json -> blocks/cta-banner/metadata.json
- component-definition.json
- component-filters.json
- component-models.json
- tools/importer/import-hey-conad.bundle.js
- tools/importer/import-hey-conad.js
- tools/importer/page-templates.json
- tools/importer/parsers/columns-banner.js
- tools/importer/parsers/cta-banner.js
- tools/importer/reports/hey-conad.report.json
- tools/importer/reports/import-hey-conad.report.xlsx
- tools/importer/transformers/conad-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-hey-conad.report.xlsx
+++ b/tools/importer/reports/import-hey-conad.report.xlsx
@@ -40,7 +40,7 @@
     <t>hey-conad.report.json</t>
   </si>
   <si>
-    <t>["hero-landing","columns-banner","promo-card","promo-card","promo-card","promo-card"]</t>
+    <t>["hero-landing","cta-banner","promo-card","promo-card","promo-card","promo-card"]</t>
   </si>
   <si>
     <t>hey-conad</t>
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-05-26T16:43:04.041Z</t>
+    <t>2026-05-26T17:11:32.759Z</t>
   </si>
   <si>
     <t>Hey Conad | Scarica l’App | Acquista Online i nostri Servizi Digitali | Conad</t>

</xml_diff>